<commit_message>
weed number stats done
</commit_message>
<xml_diff>
--- a/data/stats/supp_tables/fallcover-cc-anova.xlsx
+++ b/data/stats/supp_tables/fallcover-cc-anova.xlsx
@@ -351,26 +351,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>term</t>
+          <t>model term</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>statistic</t>
+          <t>df1</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>df</t>
+          <t>df2</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>F.ratio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Chisq</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>p.value</t>
         </is>
@@ -383,13 +393,21 @@
         </is>
       </c>
       <c r="B2">
-        <v>2.471910437076554</v>
-      </c>
-      <c r="C2">
         <v>2</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D2">
-        <v>0.2905570842540172</v>
+        <v>1.33</v>
+      </c>
+      <c r="E2">
+        <v>2.66</v>
+      </c>
+      <c r="F2">
+        <v>0.2645892429994832</v>
       </c>
     </row>
     <row r="3">
@@ -399,13 +417,21 @@
         </is>
       </c>
       <c r="B3">
-        <v>892.471999725907</v>
-      </c>
-      <c r="C3">
         <v>4</v>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D3">
-        <v>7.123679752513826E-192</v>
+        <v>254.747</v>
+      </c>
+      <c r="E3">
+        <v>1018.988</v>
+      </c>
+      <c r="F3">
+        <v>2.740698627067196E-219</v>
       </c>
     </row>
     <row r="4">
@@ -415,13 +441,21 @@
         </is>
       </c>
       <c r="B4">
-        <v>2.578508139192593</v>
-      </c>
-      <c r="C4">
         <v>1</v>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D4">
-        <v>0.1083237121588163</v>
+        <v>2.662</v>
+      </c>
+      <c r="E4">
+        <v>2.662</v>
+      </c>
+      <c r="F4">
+        <v>0.1027749986989869</v>
       </c>
     </row>
     <row r="5">
@@ -431,13 +465,21 @@
         </is>
       </c>
       <c r="B5">
-        <v>118.5160467430568</v>
-      </c>
-      <c r="C5">
         <v>1</v>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D5">
-        <v>1.336683999434482E-27</v>
+        <v>221.23</v>
+      </c>
+      <c r="E5">
+        <v>221.23</v>
+      </c>
+      <c r="F5">
+        <v>4.877026871664119E-50</v>
       </c>
     </row>
     <row r="6">
@@ -447,13 +489,21 @@
         </is>
       </c>
       <c r="B6">
-        <v>39.18643625636096</v>
-      </c>
-      <c r="C6">
         <v>8</v>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D6">
-        <v>4.538946665990326E-06</v>
+        <v>5.593</v>
+      </c>
+      <c r="E6">
+        <v>44.744</v>
+      </c>
+      <c r="F6">
+        <v>4.114191462409115E-07</v>
       </c>
     </row>
     <row r="7">
@@ -463,45 +513,69 @@
         </is>
       </c>
       <c r="B7">
-        <v>1.685006804156964</v>
-      </c>
-      <c r="C7">
         <v>2</v>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D7">
-        <v>0.4306311300489555</v>
+        <v>1.388</v>
+      </c>
+      <c r="E7">
+        <v>2.776</v>
+      </c>
+      <c r="F7">
+        <v>0.2496396067753656</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cctrt_id:straw_id</t>
+          <t>till_id:weayear</t>
         </is>
       </c>
       <c r="B8">
-        <v>7.587283841662838</v>
-      </c>
-      <c r="C8">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
       </c>
       <c r="D8">
-        <v>0.1079214662413471</v>
+        <v>2.576</v>
+      </c>
+      <c r="E8">
+        <v>5.152</v>
+      </c>
+      <c r="F8">
+        <v>0.07604249615264</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>till_id:weayear</t>
+          <t>cctrt_id:straw_id</t>
         </is>
       </c>
       <c r="B9">
-        <v>8.366122460501833</v>
-      </c>
-      <c r="C9">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
       </c>
       <c r="D9">
-        <v>0.0152517469216357</v>
+        <v>2.058</v>
+      </c>
+      <c r="E9">
+        <v>8.231999999999999</v>
+      </c>
+      <c r="F9">
+        <v>0.08349072992330604</v>
       </c>
     </row>
     <row r="10">
@@ -511,13 +585,21 @@
         </is>
       </c>
       <c r="B10">
-        <v>399.0516501060099</v>
-      </c>
-      <c r="C10">
         <v>4</v>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D10">
-        <v>4.45867168500483E-85</v>
+        <v>108.812</v>
+      </c>
+      <c r="E10">
+        <v>435.248</v>
+      </c>
+      <c r="F10">
+        <v>6.705252052934674E-93</v>
       </c>
     </row>
     <row r="11">
@@ -527,13 +609,21 @@
         </is>
       </c>
       <c r="B11">
-        <v>4.605379130842781</v>
-      </c>
-      <c r="C11">
         <v>1</v>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D11">
-        <v>0.03187180519884122</v>
+        <v>4.376</v>
+      </c>
+      <c r="E11">
+        <v>4.376</v>
+      </c>
+      <c r="F11">
+        <v>0.03644654436681943</v>
       </c>
     </row>
     <row r="12">
@@ -543,13 +633,21 @@
         </is>
       </c>
       <c r="B12">
-        <v>4.999591165889824</v>
-      </c>
-      <c r="C12">
         <v>8</v>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D12">
-        <v>0.7576198290461678</v>
+        <v>0.849</v>
+      </c>
+      <c r="E12">
+        <v>6.792</v>
+      </c>
+      <c r="F12">
+        <v>0.5591096336815535</v>
       </c>
     </row>
     <row r="13">
@@ -559,13 +657,21 @@
         </is>
       </c>
       <c r="B13">
-        <v>55.98414923727209</v>
-      </c>
-      <c r="C13">
         <v>8</v>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D13">
-        <v>2.840965088692911E-09</v>
+        <v>7.107</v>
+      </c>
+      <c r="E13">
+        <v>56.856</v>
+      </c>
+      <c r="F13">
+        <v>1.92260348034585E-09</v>
       </c>
     </row>
     <row r="14">
@@ -575,13 +681,21 @@
         </is>
       </c>
       <c r="B14">
-        <v>3.499648436394301</v>
-      </c>
-      <c r="C14">
         <v>2</v>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D14">
-        <v>0.173804492432412</v>
+        <v>2.368</v>
+      </c>
+      <c r="E14">
+        <v>4.736</v>
+      </c>
+      <c r="F14">
+        <v>0.09368265645391015</v>
       </c>
     </row>
     <row r="15">
@@ -591,13 +705,21 @@
         </is>
       </c>
       <c r="B15">
-        <v>10.55648558892486</v>
-      </c>
-      <c r="C15">
         <v>4</v>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D15">
-        <v>0.03202774684644819</v>
+        <v>2.187</v>
+      </c>
+      <c r="E15">
+        <v>8.747999999999999</v>
+      </c>
+      <c r="F15">
+        <v>0.06770877588056823</v>
       </c>
     </row>
     <row r="16">
@@ -607,13 +729,21 @@
         </is>
       </c>
       <c r="B16">
-        <v>13.22442078448144</v>
-      </c>
-      <c r="C16">
         <v>8</v>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Inf</t>
+        </is>
+      </c>
       <c r="D16">
-        <v>0.1043577389722225</v>
+        <v>1.653</v>
+      </c>
+      <c r="E16">
+        <v>13.224</v>
+      </c>
+      <c r="F16">
+        <v>0.1043577389722224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>